<commit_message>
add: Supervisor & OT Group import/export
</commit_message>
<xml_diff>
--- a/server/templates/employee-template.xlsx
+++ b/server/templates/employee-template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Documents\projects\nanafruit-hrm\server\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD648A8D-A959-4F0A-9C0D-98303BA531A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E163F3F6-F101-4FC1-8E59-E57E7918C525}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="35">
   <si>
     <t>รหัสลายนิ้วมือ</t>
   </si>
@@ -285,6 +285,18 @@
   </si>
   <si>
     <t>EMP-IMP</t>
+  </si>
+  <si>
+    <t>หัวหน้างาน</t>
+  </si>
+  <si>
+    <t>EMPCODE001</t>
+  </si>
+  <si>
+    <t>กลุ่ม OT</t>
+  </si>
+  <si>
+    <t>OT Normal</t>
   </si>
 </sst>
 </file>
@@ -708,7 +720,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="24" x14ac:dyDescent="0.55000000000000004"/>
   <cols>
     <col min="1" max="1" width="15.5703125" style="3" customWidth="1"/>
@@ -721,21 +733,22 @@
     <col min="8" max="8" width="11.42578125" style="3" customWidth="1"/>
     <col min="9" max="9" width="19.7109375" style="3" customWidth="1"/>
     <col min="10" max="10" width="20.28515625" style="3" customWidth="1"/>
-    <col min="11" max="12" width="17.28515625" style="3" customWidth="1"/>
-    <col min="13" max="13" width="21.140625" style="3" customWidth="1"/>
-    <col min="14" max="14" width="16.5703125" style="3" customWidth="1"/>
-    <col min="15" max="15" width="17.85546875" style="3" customWidth="1"/>
-    <col min="16" max="16" width="19.85546875" style="3" customWidth="1"/>
-    <col min="17" max="17" width="20.140625" style="3" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="3"/>
+    <col min="11" max="13" width="17.28515625" style="3" customWidth="1"/>
+    <col min="14" max="14" width="21.140625" style="3" customWidth="1"/>
+    <col min="15" max="15" width="16.5703125" style="3" customWidth="1"/>
+    <col min="16" max="16" width="17.85546875" style="3" customWidth="1"/>
+    <col min="17" max="17" width="19.85546875" style="3" customWidth="1"/>
+    <col min="18" max="18" width="20.140625" style="3" customWidth="1"/>
+    <col min="19" max="19" width="19.85546875" style="3" customWidth="1"/>
+    <col min="20" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.55000000000000004">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A1" s="7" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="2" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.55000000000000004">
+    <row r="2" spans="1:19" s="1" customFormat="1" x14ac:dyDescent="0.55000000000000004">
       <c r="A2" s="8" t="s">
         <v>4</v>
       </c>
@@ -773,22 +786,28 @@
         <v>28</v>
       </c>
       <c r="M2" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="N2" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="N2" s="8" t="s">
+      <c r="O2" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="O2" s="8" t="s">
+      <c r="P2" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="P2" s="8" t="s">
+      <c r="Q2" s="8" t="s">
         <v>3</v>
       </c>
-      <c r="Q2" s="8" t="s">
+      <c r="R2" s="8" t="s">
         <v>15</v>
       </c>
+      <c r="S2" s="8" t="s">
+        <v>33</v>
+      </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.55000000000000004">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.55000000000000004">
       <c r="A3" s="4" t="s">
         <v>16</v>
       </c>
@@ -826,19 +845,25 @@
         <v>29</v>
       </c>
       <c r="M3" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="N3" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="N3" s="4" t="s">
+      <c r="O3" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="O3" s="4" t="s">
+      <c r="P3" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="P3" s="4" t="s">
+      <c r="Q3" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="Q3" s="4" t="s">
+      <c r="R3" s="4" t="s">
         <v>26</v>
+      </c>
+      <c r="S3" s="4" t="s">
+        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>